<commit_message>
final not normalized fitness
</commit_message>
<xml_diff>
--- a/experiment/Final Eksperimen/Model1/best_per_run.xlsx
+++ b/experiment/Final Eksperimen/Model1/best_per_run.xlsx
@@ -502,12 +502,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>0.00000626</t>
+          <t>159750.00000000</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>237.32s</t>
+          <t>288.57s</t>
         </is>
       </c>
     </row>
@@ -526,12 +526,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>0.00000630</t>
+          <t>158710.00000000</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>230.29s</t>
+          <t>272.9s</t>
         </is>
       </c>
     </row>
@@ -550,12 +550,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0.00000627</t>
+          <t>159470.00000000</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>203.35s</t>
+          <t>264.94s</t>
         </is>
       </c>
     </row>
@@ -574,12 +574,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>0.00000619</t>
+          <t>161450.00000000</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>203.6s</t>
+          <t>273.23s</t>
         </is>
       </c>
     </row>
@@ -598,12 +598,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>0.00000626</t>
+          <t>159740.00000000</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>202.73s</t>
+          <t>249.23s</t>
         </is>
       </c>
     </row>
@@ -622,12 +622,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>0.00000643</t>
+          <t>155520.00000000</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>624.3s</t>
+          <t>728.45s</t>
         </is>
       </c>
     </row>
@@ -646,12 +646,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0.00000650</t>
+          <t>153810.00000000</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>684.95s</t>
+          <t>724.93s</t>
         </is>
       </c>
     </row>
@@ -670,12 +670,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>0.00000646</t>
+          <t>154820.00000000</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>690.59s</t>
+          <t>762.2s</t>
         </is>
       </c>
     </row>
@@ -694,12 +694,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>0.00000655</t>
+          <t>152760.00000000</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>676.05s</t>
+          <t>678.74s</t>
         </is>
       </c>
     </row>
@@ -718,12 +718,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>0.00000677</t>
+          <t>147670.00000000</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>700.33s</t>
+          <t>660.93s</t>
         </is>
       </c>
     </row>
@@ -742,12 +742,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>0.00000643</t>
+          <t>155520.00000000</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>993.36s</t>
+          <t>1243.2s</t>
         </is>
       </c>
     </row>
@@ -766,12 +766,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>0.00000672</t>
+          <t>148830.00000000</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>1035.16s</t>
+          <t>1361.21s</t>
         </is>
       </c>
     </row>
@@ -790,12 +790,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>0.00000682</t>
+          <t>146710.00000000</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>1088.36s</t>
+          <t>1234.74s</t>
         </is>
       </c>
     </row>
@@ -814,12 +814,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>0.00000682</t>
+          <t>146540.00000000</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>1088.04s</t>
+          <t>1085.76s</t>
         </is>
       </c>
     </row>
@@ -838,12 +838,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>0.00000677</t>
+          <t>147670.00000000</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>1061.52s</t>
+          <t>1088.45s</t>
         </is>
       </c>
     </row>
@@ -862,12 +862,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>0.00000686</t>
+          <t>145780.00000000</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>1959.14s</t>
+          <t>2170.62s</t>
         </is>
       </c>
     </row>
@@ -886,12 +886,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>0.00000691</t>
+          <t>144730.00000000</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2172.57s</t>
+          <t>2182.43s</t>
         </is>
       </c>
     </row>
@@ -910,12 +910,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>0.00000692</t>
+          <t>144540.00000000</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2081.51s</t>
+          <t>2182.12s</t>
         </is>
       </c>
     </row>
@@ -934,12 +934,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>0.00000687</t>
+          <t>145560.00000000</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2062.65s</t>
+          <t>2173.84s</t>
         </is>
       </c>
     </row>
@@ -958,12 +958,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>0.00000678</t>
+          <t>147480.00000000</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2058.96s</t>
+          <t>2180.45s</t>
         </is>
       </c>
     </row>
@@ -982,12 +982,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>0.00000626</t>
+          <t>159810.00000000</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>351.49s</t>
+          <t>371.88s</t>
         </is>
       </c>
     </row>
@@ -1006,12 +1006,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>0.00000669</t>
+          <t>149530.00000000</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>351.48s</t>
+          <t>371.31s</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>0.00000614</t>
+          <t>162820.00000000</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>355.3s</t>
+          <t>375.49s</t>
         </is>
       </c>
     </row>
@@ -1054,12 +1054,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>0.00000618</t>
+          <t>161850.00000000</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>357.48s</t>
+          <t>369.61s</t>
         </is>
       </c>
     </row>
@@ -1078,12 +1078,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>0.00000642</t>
+          <t>155720.00000000</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>336.68s</t>
+          <t>372.71s</t>
         </is>
       </c>
     </row>
@@ -1102,12 +1102,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>0.00000663</t>
+          <t>150810.00000000</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>992.47s</t>
+          <t>1102.31s</t>
         </is>
       </c>
     </row>
@@ -1126,12 +1126,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>0.00000669</t>
+          <t>149530.00000000</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>1067.57s</t>
+          <t>1094.0s</t>
         </is>
       </c>
     </row>
@@ -1150,12 +1150,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>0.00000651</t>
+          <t>153610.00000000</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>1123.16s</t>
+          <t>1094.64s</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1174,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>0.00000667</t>
+          <t>149860.00000000</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>1105.25s</t>
+          <t>1084.5s</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>0.00000669</t>
+          <t>149550.00000000</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>1034.06s</t>
+          <t>1081.8s</t>
         </is>
       </c>
     </row>
@@ -1222,12 +1222,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>0.00000663</t>
+          <t>150780.00000000</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>1724.06s</t>
+          <t>1804.05s</t>
         </is>
       </c>
     </row>
@@ -1246,12 +1246,12 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>0.00000696</t>
+          <t>143600.00000000</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>1736.27s</t>
+          <t>1787.9s</t>
         </is>
       </c>
     </row>
@@ -1270,12 +1270,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>0.00000669</t>
+          <t>149500.00000000</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>1900.18s</t>
+          <t>1805.58s</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>0.00000683</t>
+          <t>146470.00000000</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>1712.03s</t>
+          <t>1799.0s</t>
         </is>
       </c>
     </row>
@@ -1318,12 +1318,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>0.00000707</t>
+          <t>141500.00000000</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>1776.83s</t>
+          <t>1798.1s</t>
         </is>
       </c>
     </row>
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>0.00000686</t>
+          <t>145800.00000000</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>3463.45s</t>
+          <t>3595.14s</t>
         </is>
       </c>
     </row>
@@ -1366,12 +1366,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>0.00000696</t>
+          <t>143600.00000000</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>3377.46s</t>
+          <t>3584.9s</t>
         </is>
       </c>
     </row>
@@ -1390,12 +1390,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>0.00000696</t>
+          <t>143600.00000000</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>3609.07s</t>
+          <t>3607.71s</t>
         </is>
       </c>
     </row>
@@ -1414,12 +1414,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>0.00000710</t>
+          <t>140860.00000000</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>3702.61s</t>
+          <t>3997.11s</t>
         </is>
       </c>
     </row>
@@ -1438,12 +1438,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>0.00000707</t>
+          <t>141500.00000000</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>3541.92s</t>
+          <t>4294.37s</t>
         </is>
       </c>
     </row>

</xml_diff>